<commit_message>
remove unknowns for air location,
</commit_message>
<xml_diff>
--- a/inst/extdata/Table 1. ECHO Kits and Aliquots.xlsx
+++ b/inst/extdata/Table 1. ECHO Kits and Aliquots.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29421"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vumc365.sharepoint.com/sites/ELVISLabCore/Receiving Accessioning and Biobanking/Biostore Projection Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eric/Documents/biostoreCapacity/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E12499FA-8CA2-460B-BB78-6BBF4CF6AACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4878EB08-4B6B-6A44-BD91-8D48212B4966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38200" yWindow="500" windowWidth="40860" windowHeight="21100" firstSheet="7" activeTab="1" xr2:uid="{F4C74B1F-0A1C-8C43-884D-C02F119AE55F}"/>
+    <workbookView xWindow="-38400" yWindow="500" windowWidth="38400" windowHeight="20420" firstSheet="1" activeTab="1" xr2:uid="{F4C74B1F-0A1C-8C43-884D-C02F119AE55F}"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1. ECHO Kits and Labware" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="858" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="155">
   <si>
     <t>Protocol Version</t>
   </si>
@@ -1013,19 +1013,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3D8EFBD-9C1F-B14B-B50F-F1873B963E4E}">
   <dimension ref="A1:J46"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.85546875" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" style="3"/>
-    <col min="6" max="6" width="21.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" style="3"/>
+    <col min="6" max="6" width="21.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" ht="41.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="42">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1603,7 +1603,7 @@
         <v>24</v>
       </c>
       <c r="H19" s="3">
-        <f>7*4</f>
+        <f t="shared" ref="H19:H37" si="1">7*4</f>
         <v>28</v>
       </c>
       <c r="I19">
@@ -1634,7 +1634,7 @@
         <v>24</v>
       </c>
       <c r="H20" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I20">
@@ -1665,7 +1665,7 @@
         <v>24</v>
       </c>
       <c r="H21" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I21">
@@ -1696,7 +1696,7 @@
         <v>24</v>
       </c>
       <c r="H22" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I22">
@@ -1727,7 +1727,7 @@
         <v>24</v>
       </c>
       <c r="H23" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I23">
@@ -1758,7 +1758,7 @@
         <v>96</v>
       </c>
       <c r="H24" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I24">
@@ -1789,7 +1789,7 @@
         <v>96</v>
       </c>
       <c r="H25" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I25">
@@ -1820,7 +1820,7 @@
         <v>96</v>
       </c>
       <c r="H26" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I26">
@@ -1851,7 +1851,7 @@
         <v>96</v>
       </c>
       <c r="H27" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I27">
@@ -1882,7 +1882,7 @@
         <v>48</v>
       </c>
       <c r="H28" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I28">
@@ -1913,7 +1913,7 @@
         <v>48</v>
       </c>
       <c r="H29" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I29">
@@ -1944,7 +1944,7 @@
         <v>48</v>
       </c>
       <c r="H30" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I30">
@@ -1975,7 +1975,7 @@
         <v>48</v>
       </c>
       <c r="H31" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I31">
@@ -2006,7 +2006,7 @@
         <v>48</v>
       </c>
       <c r="H32" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I32">
@@ -2037,7 +2037,7 @@
         <v>48</v>
       </c>
       <c r="H33" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I33">
@@ -2068,7 +2068,7 @@
         <v>48</v>
       </c>
       <c r="H34" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I34">
@@ -2099,7 +2099,7 @@
         <v>48</v>
       </c>
       <c r="H35" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I35">
@@ -2130,7 +2130,7 @@
         <v>48</v>
       </c>
       <c r="H36" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I36">
@@ -2161,7 +2161,7 @@
         <v>48</v>
       </c>
       <c r="H37" s="3">
-        <f>7*4</f>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="I37">
@@ -2255,7 +2255,7 @@
         <v>24</v>
       </c>
       <c r="H40" s="3">
-        <f>7*4</f>
+        <f t="shared" ref="H40:H46" si="2">7*4</f>
         <v>28</v>
       </c>
       <c r="I40">
@@ -2286,7 +2286,7 @@
         <v>96</v>
       </c>
       <c r="H41" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I41">
@@ -2317,7 +2317,7 @@
         <v>96</v>
       </c>
       <c r="H42" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I42">
@@ -2348,7 +2348,7 @@
         <v>96</v>
       </c>
       <c r="H43" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I43">
@@ -2379,7 +2379,7 @@
         <v>48</v>
       </c>
       <c r="H44" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I44">
@@ -2410,7 +2410,7 @@
         <v>48</v>
       </c>
       <c r="H45" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I45">
@@ -2441,7 +2441,7 @@
         <v>48</v>
       </c>
       <c r="H46" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I46">
@@ -2463,21 +2463,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7139A15E-63C2-4CF1-A0FB-2A52DEBA8541}">
   <dimension ref="A1:J54"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="31.28515625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.5703125" style="3" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="9.42578125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="9.28515625" style="3" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" customWidth="1"/>
-    <col min="10" max="10" width="31.28515625" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5" style="3" customWidth="1"/>
+    <col min="5" max="5" width="11.5" style="3" customWidth="1"/>
+    <col min="6" max="6" width="21.1640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="9.5" style="3" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" style="3" customWidth="1"/>
+    <col min="9" max="9" width="11.5" customWidth="1"/>
+    <col min="10" max="10" width="31.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" ht="41.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" ht="42">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2536,7 +2536,7 @@
         <v>20</v>
       </c>
       <c r="I2">
-        <f>G2*H2</f>
+        <f t="shared" ref="I2:I33" si="0">G2*H2</f>
         <v>1400</v>
       </c>
       <c r="J2" t="s">
@@ -2571,7 +2571,7 @@
         <v>20</v>
       </c>
       <c r="I3">
-        <f>G3*H3</f>
+        <f t="shared" si="0"/>
         <v>720</v>
       </c>
       <c r="J3" t="s">
@@ -2605,7 +2605,7 @@
         <v>28</v>
       </c>
       <c r="I4">
-        <f>G4*H4</f>
+        <f t="shared" si="0"/>
         <v>2688</v>
       </c>
       <c r="J4" t="s">
@@ -2639,7 +2639,7 @@
         <v>28</v>
       </c>
       <c r="I5">
-        <f>G5*H5</f>
+        <f t="shared" si="0"/>
         <v>1344</v>
       </c>
       <c r="J5" t="s">
@@ -2673,7 +2673,7 @@
         <v>20</v>
       </c>
       <c r="I6">
-        <f>G6*H6</f>
+        <f t="shared" si="0"/>
         <v>1400</v>
       </c>
       <c r="J6" s="3" t="s">
@@ -2707,7 +2707,7 @@
         <v>20</v>
       </c>
       <c r="I7">
-        <f>G7*H7</f>
+        <f t="shared" si="0"/>
         <v>1400</v>
       </c>
       <c r="J7" s="3" t="s">
@@ -2741,7 +2741,7 @@
         <v>20</v>
       </c>
       <c r="I8">
-        <f>G8*H8</f>
+        <f t="shared" si="0"/>
         <v>1400</v>
       </c>
       <c r="J8" s="3" t="s">
@@ -2775,7 +2775,7 @@
         <v>20</v>
       </c>
       <c r="I9">
-        <f>G9*H9</f>
+        <f t="shared" si="0"/>
         <v>1400</v>
       </c>
       <c r="J9" s="3" t="s">
@@ -2809,7 +2809,7 @@
         <v>20</v>
       </c>
       <c r="I10">
-        <f>G10*H10</f>
+        <f t="shared" si="0"/>
         <v>1400</v>
       </c>
       <c r="J10" t="s">
@@ -2843,7 +2843,7 @@
         <v>28</v>
       </c>
       <c r="I11">
-        <f>G11*H11</f>
+        <f t="shared" si="0"/>
         <v>2688</v>
       </c>
       <c r="J11" t="s">
@@ -2877,7 +2877,7 @@
         <v>28</v>
       </c>
       <c r="I12">
-        <f>G12*H12</f>
+        <f t="shared" si="0"/>
         <v>1344</v>
       </c>
       <c r="J12" t="s">
@@ -2912,7 +2912,7 @@
         <v>20</v>
       </c>
       <c r="I13">
-        <f>G13*H13</f>
+        <f t="shared" si="0"/>
         <v>980</v>
       </c>
       <c r="J13" t="s">
@@ -2947,7 +2947,7 @@
         <v>20</v>
       </c>
       <c r="I14">
-        <f>G14*H14</f>
+        <f t="shared" si="0"/>
         <v>720</v>
       </c>
       <c r="J14" t="s">
@@ -2980,7 +2980,7 @@
         <v>10</v>
       </c>
       <c r="I15">
-        <f>G15*H15</f>
+        <f t="shared" si="0"/>
         <v>160</v>
       </c>
       <c r="J15" t="s">
@@ -3014,7 +3014,7 @@
         <v>28</v>
       </c>
       <c r="I16">
-        <f>G16*H16</f>
+        <f t="shared" si="0"/>
         <v>1344</v>
       </c>
       <c r="J16" t="s">
@@ -3048,7 +3048,7 @@
         <v>20</v>
       </c>
       <c r="I17">
-        <f>G17*H17</f>
+        <f t="shared" si="0"/>
         <v>720</v>
       </c>
       <c r="J17" t="s">
@@ -3082,7 +3082,7 @@
         <v>20</v>
       </c>
       <c r="I18">
-        <f>G18*H18</f>
+        <f t="shared" si="0"/>
         <v>720</v>
       </c>
       <c r="J18" t="s">
@@ -3116,7 +3116,7 @@
         <v>20</v>
       </c>
       <c r="I19">
-        <f>G19*H19</f>
+        <f t="shared" si="0"/>
         <v>720</v>
       </c>
       <c r="J19" t="s">
@@ -3143,14 +3143,14 @@
         <v>24</v>
       </c>
       <c r="G20" s="3">
-        <f>5*5</f>
+        <f t="shared" ref="G20:G25" si="1">5*5</f>
         <v>25</v>
       </c>
       <c r="H20" s="6">
         <v>20</v>
       </c>
       <c r="I20">
-        <f>G20*H20</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="J20" t="s">
@@ -3177,14 +3177,14 @@
         <v>24</v>
       </c>
       <c r="G21" s="3">
-        <f>5*5</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="H21" s="6">
         <v>20</v>
       </c>
       <c r="I21">
-        <f>G21*H21</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="J21" t="s">
@@ -3211,14 +3211,14 @@
         <v>24</v>
       </c>
       <c r="G22" s="3">
-        <f>5*5</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="H22" s="6">
         <v>20</v>
       </c>
       <c r="I22">
-        <f>G22*H22</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="J22" t="s">
@@ -3245,14 +3245,14 @@
         <v>24</v>
       </c>
       <c r="G23" s="3">
-        <f>5*5</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="H23" s="6">
         <v>20</v>
       </c>
       <c r="I23">
-        <f>G23*H23</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="J23" t="s">
@@ -3279,14 +3279,14 @@
         <v>24</v>
       </c>
       <c r="G24" s="3">
-        <f>5*5</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="H24" s="6">
         <v>20</v>
       </c>
       <c r="I24">
-        <f>G24*H24</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="J24" t="s">
@@ -3313,14 +3313,14 @@
         <v>24</v>
       </c>
       <c r="G25" s="3">
-        <f>5*5</f>
+        <f t="shared" si="1"/>
         <v>25</v>
       </c>
       <c r="H25" s="6">
         <v>20</v>
       </c>
       <c r="I25">
-        <f>G25*H25</f>
+        <f t="shared" si="0"/>
         <v>500</v>
       </c>
       <c r="J25" t="s">
@@ -3350,11 +3350,11 @@
         <v>24</v>
       </c>
       <c r="H26" s="3">
-        <f>7*4</f>
+        <f t="shared" ref="H26:H37" si="2">7*4</f>
         <v>28</v>
       </c>
       <c r="I26">
-        <f>G26*H26</f>
+        <f t="shared" si="0"/>
         <v>672</v>
       </c>
       <c r="J26" t="s">
@@ -3384,11 +3384,11 @@
         <v>48</v>
       </c>
       <c r="H27" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I27">
-        <f>G27*H27</f>
+        <f t="shared" si="0"/>
         <v>1344</v>
       </c>
       <c r="J27" t="s">
@@ -3418,11 +3418,11 @@
         <v>24</v>
       </c>
       <c r="H28" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I28">
-        <f>G28*H28</f>
+        <f t="shared" si="0"/>
         <v>672</v>
       </c>
       <c r="J28" t="s">
@@ -3452,11 +3452,11 @@
         <v>48</v>
       </c>
       <c r="H29" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I29">
-        <f>G29*H29</f>
+        <f t="shared" si="0"/>
         <v>1344</v>
       </c>
       <c r="J29" t="s">
@@ -3486,11 +3486,11 @@
         <v>24</v>
       </c>
       <c r="H30" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I30">
-        <f>G30*H30</f>
+        <f t="shared" si="0"/>
         <v>672</v>
       </c>
       <c r="J30" t="s">
@@ -3520,11 +3520,11 @@
         <v>48</v>
       </c>
       <c r="H31" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I31">
-        <f>G31*H31</f>
+        <f t="shared" si="0"/>
         <v>1344</v>
       </c>
       <c r="J31" t="s">
@@ -3554,11 +3554,11 @@
         <v>24</v>
       </c>
       <c r="H32" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I32">
-        <f>G32*H32</f>
+        <f t="shared" si="0"/>
         <v>672</v>
       </c>
       <c r="J32" t="s">
@@ -3588,11 +3588,11 @@
         <v>48</v>
       </c>
       <c r="H33" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I33">
-        <f>G33*H33</f>
+        <f t="shared" si="0"/>
         <v>1344</v>
       </c>
       <c r="J33" t="s">
@@ -3622,11 +3622,11 @@
         <v>24</v>
       </c>
       <c r="H34" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I34">
-        <f>G34*H34</f>
+        <f t="shared" ref="I34:I65" si="3">G34*H34</f>
         <v>672</v>
       </c>
       <c r="J34" t="s">
@@ -3656,11 +3656,11 @@
         <v>48</v>
       </c>
       <c r="H35" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I35">
-        <f>G35*H35</f>
+        <f t="shared" si="3"/>
         <v>1344</v>
       </c>
       <c r="J35" t="s">
@@ -3690,11 +3690,11 @@
         <v>24</v>
       </c>
       <c r="H36" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I36">
-        <f>G36*H36</f>
+        <f t="shared" si="3"/>
         <v>672</v>
       </c>
       <c r="J36" t="s">
@@ -3724,11 +3724,11 @@
         <v>48</v>
       </c>
       <c r="H37" s="3">
-        <f>7*4</f>
+        <f t="shared" si="2"/>
         <v>28</v>
       </c>
       <c r="I37">
-        <f>G37*H37</f>
+        <f t="shared" si="3"/>
         <v>1344</v>
       </c>
       <c r="J37" t="s">
@@ -3761,7 +3761,7 @@
         <v>10</v>
       </c>
       <c r="I38">
-        <f>G38*H38</f>
+        <f t="shared" si="3"/>
         <v>160</v>
       </c>
       <c r="J38" t="s">
@@ -3795,7 +3795,7 @@
         <v>10</v>
       </c>
       <c r="I39">
-        <f>G39*H39</f>
+        <f t="shared" si="3"/>
         <v>160</v>
       </c>
       <c r="J39" t="s">
@@ -3828,7 +3828,7 @@
         <v>10</v>
       </c>
       <c r="I40">
-        <f>G40*H40</f>
+        <f t="shared" si="3"/>
         <v>160</v>
       </c>
       <c r="J40" t="s">
@@ -3856,10 +3856,6 @@
       </c>
       <c r="G41" s="3">
         <v>1</v>
-      </c>
-      <c r="I41">
-        <f>G41*H41</f>
-        <v>0</v>
       </c>
       <c r="J41" t="s">
         <v>61</v>
@@ -3892,7 +3888,7 @@
         <v>20</v>
       </c>
       <c r="I42">
-        <f>G42*H42</f>
+        <f t="shared" si="3"/>
         <v>1400</v>
       </c>
       <c r="J42" t="s">
@@ -3926,7 +3922,7 @@
         <v>28</v>
       </c>
       <c r="I43">
-        <f>G43*H43</f>
+        <f t="shared" si="3"/>
         <v>2688</v>
       </c>
       <c r="J43" t="s">
@@ -3960,7 +3956,7 @@
         <v>28</v>
       </c>
       <c r="I44">
-        <f>G44*H44</f>
+        <f t="shared" si="3"/>
         <v>1344</v>
       </c>
       <c r="J44" t="s">
@@ -3994,7 +3990,7 @@
         <v>20</v>
       </c>
       <c r="I45">
-        <f>G45*H45</f>
+        <f t="shared" si="3"/>
         <v>1400</v>
       </c>
       <c r="J45" t="s">
@@ -4028,7 +4024,7 @@
         <v>28</v>
       </c>
       <c r="I46">
-        <f>G46*H46</f>
+        <f t="shared" si="3"/>
         <v>2688</v>
       </c>
       <c r="J46" t="s">
@@ -4062,7 +4058,7 @@
         <v>28</v>
       </c>
       <c r="I47">
-        <f>G47*H47</f>
+        <f t="shared" si="3"/>
         <v>1344</v>
       </c>
       <c r="J47" t="s">
@@ -4096,7 +4092,7 @@
         <v>20</v>
       </c>
       <c r="I48">
-        <f>G48*H48</f>
+        <f t="shared" si="3"/>
         <v>1400</v>
       </c>
       <c r="J48" t="s">
@@ -4130,7 +4126,7 @@
         <v>28</v>
       </c>
       <c r="I49">
-        <f>G49*H49</f>
+        <f t="shared" si="3"/>
         <v>2688</v>
       </c>
       <c r="J49" t="s">
@@ -4164,7 +4160,7 @@
         <v>28</v>
       </c>
       <c r="I50">
-        <f>G50*H50</f>
+        <f t="shared" si="3"/>
         <v>1344</v>
       </c>
       <c r="J50" t="s">
@@ -4187,18 +4183,7 @@
       <c r="E51" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F51" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G51" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H51" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="I51" s="3" t="s">
-        <v>81</v>
-      </c>
+      <c r="I51" s="3"/>
       <c r="J51" t="s">
         <v>78</v>
       </c>
@@ -4219,18 +4204,6 @@
       <c r="E52" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F52" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G52" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H52" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="I52" t="s">
-        <v>81</v>
-      </c>
       <c r="J52" t="s">
         <v>82</v>
       </c>
@@ -4251,18 +4224,7 @@
       <c r="E53" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="F53" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="G53" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="H53" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="I53" s="3" t="s">
-        <v>81</v>
-      </c>
+      <c r="I53" s="3"/>
       <c r="J53" t="s">
         <v>83</v>
       </c>
@@ -4311,9 +4273,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4BD62B0-A2FC-D94D-A1AE-A7A7B8D015EE}">
   <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4374,7 +4336,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CB692F1-5371-7D49-88B9-1A0C085FB643}">
   <dimension ref="A2:D3"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13"/>
   <sheetData>
     <row r="2" spans="1:4" ht="15">
       <c r="A2" t="s">
@@ -4410,7 +4372,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5C04190-97A0-B648-86E7-26BDE31B3437}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="12.95"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="13"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4419,18 +4381,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63DAE0FF-453D-47E8-B705-AB8CE28B14D2}">
   <dimension ref="A1:J42"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="74.140625" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" customWidth="1"/>
-    <col min="5" max="6" width="9.140625" customWidth="1"/>
+    <col min="1" max="1" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="74.1640625" customWidth="1"/>
+    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" customWidth="1"/>
+    <col min="5" max="6" width="9.1640625" customWidth="1"/>
     <col min="7" max="7" width="34" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.42578125" customWidth="1"/>
+    <col min="10" max="10" width="18.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75">
+    <row r="1" spans="1:10" ht="17">
       <c r="A1" s="13" t="s">
         <v>95</v>
       </c>
@@ -4456,7 +4418,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.75">
+    <row r="2" spans="1:10" ht="17">
       <c r="A2" s="13" t="s">
         <v>101</v>
       </c>
@@ -4482,7 +4444,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.75">
+    <row r="3" spans="1:10" ht="17">
       <c r="A3" s="13" t="s">
         <v>101</v>
       </c>
@@ -4508,7 +4470,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.75">
+    <row r="4" spans="1:10" ht="17">
       <c r="A4" s="13" t="s">
         <v>101</v>
       </c>
@@ -4534,7 +4496,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.75">
+    <row r="5" spans="1:10" ht="17">
       <c r="A5" s="13" t="s">
         <v>101</v>
       </c>
@@ -4560,7 +4522,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.75">
+    <row r="6" spans="1:10" ht="17">
       <c r="A6" s="13" t="s">
         <v>101</v>
       </c>
@@ -4586,7 +4548,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.75">
+    <row r="7" spans="1:10" ht="17">
       <c r="A7" s="13" t="s">
         <v>101</v>
       </c>
@@ -4612,7 +4574,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15.75">
+    <row r="8" spans="1:10" ht="17">
       <c r="A8" s="13" t="s">
         <v>101</v>
       </c>
@@ -4635,7 +4597,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15.75">
+    <row r="9" spans="1:10" ht="17">
       <c r="A9" s="13" t="s">
         <v>101</v>
       </c>
@@ -4661,7 +4623,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.75">
+    <row r="10" spans="1:10" ht="17">
       <c r="A10" s="13" t="s">
         <v>101</v>
       </c>
@@ -4687,7 +4649,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15.75">
+    <row r="11" spans="1:10" ht="17">
       <c r="A11" s="13" t="s">
         <v>101</v>
       </c>
@@ -4713,7 +4675,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="15.75">
+    <row r="12" spans="1:10" ht="17">
       <c r="A12" s="13" t="s">
         <v>112</v>
       </c>
@@ -4739,7 +4701,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15.75">
+    <row r="13" spans="1:10" ht="17">
       <c r="A13" s="13" t="s">
         <v>113</v>
       </c>
@@ -4765,7 +4727,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15.75">
+    <row r="14" spans="1:10" ht="17">
       <c r="A14" s="13" t="s">
         <v>113</v>
       </c>
@@ -4791,7 +4753,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="15.75">
+    <row r="15" spans="1:10" ht="17">
       <c r="A15" s="13" t="s">
         <v>113</v>
       </c>
@@ -4817,7 +4779,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="15.75">
+    <row r="16" spans="1:10" ht="17">
       <c r="A16" s="13" t="s">
         <v>113</v>
       </c>
@@ -4843,7 +4805,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="15.75">
+    <row r="17" spans="1:10" ht="17">
       <c r="A17" s="13" t="s">
         <v>113</v>
       </c>
@@ -4869,7 +4831,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="15.75">
+    <row r="18" spans="1:10" ht="17">
       <c r="A18" s="13" t="s">
         <v>113</v>
       </c>
@@ -4893,7 +4855,7 @@
       </c>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:10" ht="15.75">
+    <row r="19" spans="1:10" ht="17">
       <c r="A19" s="13" t="s">
         <v>113</v>
       </c>
@@ -4913,7 +4875,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15.75">
+    <row r="20" spans="1:10" ht="17">
       <c r="A20" s="13" t="s">
         <v>113</v>
       </c>
@@ -4936,7 +4898,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="15.75">
+    <row r="21" spans="1:10" ht="17">
       <c r="A21" s="13" t="s">
         <v>113</v>
       </c>
@@ -4959,7 +4921,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="15.75">
+    <row r="22" spans="1:10" ht="17">
       <c r="A22" s="13" t="s">
         <v>114</v>
       </c>
@@ -4982,7 +4944,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="15.75">
+    <row r="23" spans="1:10" ht="17">
       <c r="A23" s="13" t="s">
         <v>116</v>
       </c>
@@ -5005,7 +4967,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="15.75">
+    <row r="24" spans="1:10" ht="17">
       <c r="A24" s="13" t="s">
         <v>116</v>
       </c>
@@ -5028,7 +4990,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="15.75">
+    <row r="25" spans="1:10" ht="17">
       <c r="A25" s="13" t="s">
         <v>119</v>
       </c>
@@ -5051,7 +5013,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="30.75">
+    <row r="26" spans="1:10" ht="34">
       <c r="A26" s="13" t="s">
         <v>119</v>
       </c>
@@ -5074,7 +5036,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="30.75">
+    <row r="27" spans="1:10" ht="17">
       <c r="A27" s="13" t="s">
         <v>119</v>
       </c>
@@ -5097,7 +5059,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="15.75">
+    <row r="28" spans="1:10" ht="17">
       <c r="A28" s="13" t="s">
         <v>124</v>
       </c>
@@ -5120,7 +5082,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="15.75">
+    <row r="29" spans="1:10" ht="17">
       <c r="A29" s="13" t="s">
         <v>124</v>
       </c>
@@ -5143,7 +5105,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="15.75">
+    <row r="30" spans="1:10" ht="17">
       <c r="A30" s="13" t="s">
         <v>127</v>
       </c>
@@ -5166,7 +5128,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="15.75">
+    <row r="31" spans="1:10" ht="17">
       <c r="A31" s="13" t="s">
         <v>127</v>
       </c>
@@ -5189,7 +5151,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="15.75">
+    <row r="32" spans="1:10" ht="17">
       <c r="A32" s="13" t="s">
         <v>128</v>
       </c>
@@ -5212,7 +5174,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="15.75">
+    <row r="33" spans="1:7" ht="17">
       <c r="A33" s="13" t="s">
         <v>128</v>
       </c>
@@ -5235,7 +5197,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="15.75">
+    <row r="34" spans="1:7" ht="17">
       <c r="A34" s="13" t="s">
         <v>129</v>
       </c>
@@ -5258,7 +5220,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="15.75">
+    <row r="35" spans="1:7" ht="17">
       <c r="A35" s="13" t="s">
         <v>131</v>
       </c>
@@ -5281,7 +5243,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="15.75">
+    <row r="36" spans="1:7" ht="17">
       <c r="A36" s="13" t="s">
         <v>132</v>
       </c>
@@ -5304,7 +5266,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="15.75">
+    <row r="37" spans="1:7" ht="17">
       <c r="A37" s="13" t="s">
         <v>132</v>
       </c>
@@ -5327,7 +5289,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="15.75">
+    <row r="38" spans="1:7" ht="17">
       <c r="A38" s="13" t="s">
         <v>133</v>
       </c>
@@ -5350,7 +5312,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="15.75">
+    <row r="39" spans="1:7" ht="17">
       <c r="A39" s="13" t="s">
         <v>135</v>
       </c>
@@ -5373,7 +5335,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="15.75">
+    <row r="40" spans="1:7" ht="17">
       <c r="A40" s="13" t="s">
         <v>135</v>
       </c>
@@ -5396,7 +5358,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="15.75">
+    <row r="41" spans="1:7" ht="17">
       <c r="A41" s="13" t="s">
         <v>138</v>
       </c>
@@ -5419,7 +5381,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="15.75">
+    <row r="42" spans="1:7" ht="17">
       <c r="A42" s="13" t="s">
         <v>138</v>
       </c>
@@ -5450,19 +5412,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF3ADB56-0CF8-4762-89DC-5F7DB272040A}">
   <dimension ref="A1:H34"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="37.28515625" customWidth="1"/>
-    <col min="2" max="2" width="84.140625" customWidth="1"/>
-    <col min="3" max="3" width="24.7109375" customWidth="1"/>
-    <col min="4" max="4" width="23.7109375" customWidth="1"/>
-    <col min="5" max="5" width="28.42578125" customWidth="1"/>
-    <col min="6" max="6" width="29.5703125" customWidth="1"/>
+    <col min="1" max="1" width="37.33203125" customWidth="1"/>
+    <col min="2" max="2" width="84.1640625" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
+    <col min="4" max="4" width="23.6640625" customWidth="1"/>
+    <col min="5" max="5" width="28.5" customWidth="1"/>
+    <col min="6" max="6" width="29.5" customWidth="1"/>
     <col min="7" max="7" width="17" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="32.25">
+    <row r="1" spans="1:8" ht="17">
       <c r="A1" s="13" t="s">
         <v>95</v>
       </c>
@@ -5488,7 +5450,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="16.5">
+    <row r="2" spans="1:8" ht="17">
       <c r="A2" s="16" t="s">
         <v>101</v>
       </c>
@@ -5516,7 +5478,7 @@
         <v>9148</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="16.5">
+    <row r="3" spans="1:8" ht="17">
       <c r="A3" s="16" t="s">
         <v>101</v>
       </c>
@@ -5542,7 +5504,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="16.5">
+    <row r="4" spans="1:8" ht="17">
       <c r="A4" s="16" t="s">
         <v>101</v>
       </c>
@@ -5562,15 +5524,15 @@
         <v>24862</v>
       </c>
       <c r="G4">
-        <f t="shared" ref="G3:G34" si="0">D4-E4</f>
+        <f t="shared" ref="G4:G34" si="0">D4-E4</f>
         <v>14566</v>
       </c>
       <c r="H4">
-        <f t="shared" ref="H3:H34" si="1">D4-F4</f>
+        <f t="shared" ref="H4:H34" si="1">D4-F4</f>
         <v>14568</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="16.5">
+    <row r="5" spans="1:8" ht="17">
       <c r="A5" s="16" t="s">
         <v>101</v>
       </c>
@@ -5598,7 +5560,7 @@
         <v>9840</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="16.5">
+    <row r="6" spans="1:8" ht="17">
       <c r="A6" s="16" t="s">
         <v>101</v>
       </c>
@@ -5626,7 +5588,7 @@
         <v>9205</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="16.5">
+    <row r="7" spans="1:8" ht="17">
       <c r="A7" s="16" t="s">
         <v>101</v>
       </c>
@@ -5652,7 +5614,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="16.5">
+    <row r="8" spans="1:8" ht="17">
       <c r="A8" s="16" t="s">
         <v>101</v>
       </c>
@@ -5680,7 +5642,7 @@
         <v>27842</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="16.5">
+    <row r="9" spans="1:8" ht="17">
       <c r="A9" s="16" t="s">
         <v>101</v>
       </c>
@@ -5708,7 +5670,7 @@
         <v>12418</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="16.5">
+    <row r="10" spans="1:8" ht="17">
       <c r="A10" s="16" t="s">
         <v>101</v>
       </c>
@@ -5736,7 +5698,7 @@
         <v>3385</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="16.5">
+    <row r="11" spans="1:8" ht="17">
       <c r="A11" s="16" t="s">
         <v>101</v>
       </c>
@@ -5764,7 +5726,7 @@
         <v>2284</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="16.5">
+    <row r="12" spans="1:8" ht="17">
       <c r="A12" s="16" t="s">
         <v>101</v>
       </c>
@@ -5792,7 +5754,7 @@
         <v>9287</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="16.5">
+    <row r="13" spans="1:8" ht="17">
       <c r="A13" s="16" t="s">
         <v>101</v>
       </c>
@@ -5820,7 +5782,7 @@
         <v>7630</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="16.5">
+    <row r="14" spans="1:8" ht="17">
       <c r="A14" s="16" t="s">
         <v>112</v>
       </c>
@@ -5848,7 +5810,7 @@
         <v>3138</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="16.5">
+    <row r="15" spans="1:8" ht="17">
       <c r="A15" s="16" t="s">
         <v>113</v>
       </c>
@@ -5876,7 +5838,7 @@
         <v>1663</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="16.5">
+    <row r="16" spans="1:8" ht="17">
       <c r="A16" s="16" t="s">
         <v>113</v>
       </c>
@@ -5904,7 +5866,7 @@
         <v>1900</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="16.5">
+    <row r="17" spans="1:8" ht="17">
       <c r="A17" s="16" t="s">
         <v>113</v>
       </c>
@@ -5932,7 +5894,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="16.5">
+    <row r="18" spans="1:8" ht="17">
       <c r="A18" s="16" t="s">
         <v>113</v>
       </c>
@@ -5960,7 +5922,7 @@
         <v>1733</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="16.5">
+    <row r="19" spans="1:8" ht="17">
       <c r="A19" s="16" t="s">
         <v>113</v>
       </c>
@@ -5988,7 +5950,7 @@
         <v>4429</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="16.5">
+    <row r="20" spans="1:8" ht="17">
       <c r="A20" s="16" t="s">
         <v>113</v>
       </c>
@@ -6016,7 +5978,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="16.5">
+    <row r="21" spans="1:8" ht="17">
       <c r="A21" s="16" t="s">
         <v>113</v>
       </c>
@@ -6044,7 +6006,7 @@
         <v>923</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="16.5">
+    <row r="22" spans="1:8" ht="17">
       <c r="A22" s="16" t="s">
         <v>113</v>
       </c>
@@ -6072,7 +6034,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="16.5">
+    <row r="23" spans="1:8" ht="17">
       <c r="A23" s="16" t="s">
         <v>113</v>
       </c>
@@ -6100,7 +6062,7 @@
         <v>2019</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="16.5">
+    <row r="24" spans="1:8" ht="17">
       <c r="A24" s="16" t="s">
         <v>113</v>
       </c>
@@ -6128,7 +6090,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="16.5">
+    <row r="25" spans="1:8" ht="17">
       <c r="A25" s="16" t="s">
         <v>114</v>
       </c>
@@ -6156,7 +6118,7 @@
         <v>3120</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="16.5">
+    <row r="26" spans="1:8" ht="17">
       <c r="A26" s="16" t="s">
         <v>119</v>
       </c>
@@ -6184,7 +6146,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="32.25">
+    <row r="27" spans="1:8" ht="34">
       <c r="A27" s="16" t="s">
         <v>119</v>
       </c>
@@ -6212,7 +6174,7 @@
         <v>4196</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="16.5">
+    <row r="28" spans="1:8" ht="17">
       <c r="A28" s="16" t="s">
         <v>119</v>
       </c>
@@ -6240,7 +6202,7 @@
         <v>4244</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="16.5">
+    <row r="29" spans="1:8" ht="17">
       <c r="A29" s="16" t="s">
         <v>153</v>
       </c>
@@ -6268,7 +6230,7 @@
         <v>1116</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="16.5">
+    <row r="30" spans="1:8" ht="17">
       <c r="A30" s="16" t="s">
         <v>132</v>
       </c>
@@ -6296,7 +6258,7 @@
         <v>4685</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="16.5">
+    <row r="31" spans="1:8" ht="17">
       <c r="A31" s="16" t="s">
         <v>132</v>
       </c>
@@ -6324,7 +6286,7 @@
         <v>2661</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="16.5">
+    <row r="32" spans="1:8" ht="17">
       <c r="A32" s="16" t="s">
         <v>133</v>
       </c>
@@ -6352,7 +6314,7 @@
         <v>1988</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="16.5">
+    <row r="33" spans="1:8" ht="17">
       <c r="A33" s="16" t="s">
         <v>154</v>
       </c>
@@ -6380,7 +6342,7 @@
         <v>44621</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="16.5">
+    <row r="34" spans="1:8" ht="17">
       <c r="A34" s="16" t="s">
         <v>154</v>
       </c>
@@ -6416,14 +6378,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{145477D5-2817-49CF-8DCC-FF548793A576}">
   <dimension ref="A1:F11"/>
-  <sheetFormatPr defaultRowHeight="12.75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -6652,6 +6614,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100197640FEAACA944E9F49A9EC3E91143D" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1218410fc0fa077fead1b1e9d0b3fb3c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f0b1a4ef-869e-4fa8-a4a9-08ab0e4fb563" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="c75d7b4b85ea32f677dcae992f242353" ns2:_="">
     <xsd:import namespace="f0b1a4ef-869e-4fa8-a4a9-08ab0e4fb563"/>
@@ -6813,29 +6790,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0CC95EF8-9865-4C6C-8EE2-D29DB694167F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1862DB38-2816-4165-A089-383680BAA181}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8987BF9-4E08-4D9D-BE86-2E978020A1C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E8987BF9-4E08-4D9D-BE86-2E978020A1C5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1862DB38-2816-4165-A089-383680BAA181}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0CC95EF8-9865-4C6C-8EE2-D29DB694167F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f0b1a4ef-869e-4fa8-a4a9-08ab0e4fb563"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>